<commit_message>
Agregué pruebas API y capturas
</commit_message>
<xml_diff>
--- a/bugs/reporte_bugs.xlsx
+++ b/bugs/reporte_bugs.xlsx
@@ -1,16 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brenr\OneDrive\Desktop\Bren\ADA\QA TESTING\ProyectoFinal-Ruejas\bugs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F8DF1EE-E938-43CA-999F-7197EEA79976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -20,12 +25,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Autoría desconocida</author>
   </authors>
   <commentList>
-    <comment ref="J3" authorId="0">
+    <comment ref="J3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -33,11 +38,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Sugerencia: visualización de requisitos como leyenda debajo del campo Nombre de perfil previo al ingreso de cualquier caracter permite al usuario agilizar tiempos en la creación del perfil</t>
+          <t>Sugerencia: visualización de requisitos como leyenda debajo del campo Nombre de perfil previo al ingreso de cualquier caracter permite al usuario agilizar tiempos en la creación del perfil</t>
         </r>
       </text>
     </comment>
-    <comment ref="J4" authorId="0">
+    <comment ref="J4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -45,7 +50,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Sugerencia: la corrección de este bug evita la pérdida de creación de contenido si el usuario no concretó la publicación, sin verse obligado a iniciarla nuevamente y ahorrando tiempo para volver a seleccionar, editar, mejorar y personalizar la misma</t>
+          <t>Sugerencia: la corrección de este bug evita la pérdida de creación de contenido si el usuario no concretó la publicación, sin verse obligado a iniciarla nuevamente y ahorrando tiempo para volver a seleccionar, editar, mejorar y personalizar la misma</t>
         </r>
       </text>
     </comment>
@@ -56,40 +61,40 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
   <si>
-    <t xml:space="preserve">ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descripción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Datos de Entrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pasos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resultado Esperado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resultado Obtenido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prioridad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Severidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observaciones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Límite de intentos de edición del Nombre de perfil (1 vez cada 7 días)</t>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Datos de Entrada</t>
+  </si>
+  <si>
+    <t>Pasos</t>
+  </si>
+  <si>
+    <t>Resultado Esperado</t>
+  </si>
+  <si>
+    <t>Resultado Obtenido</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Prioridad</t>
+  </si>
+  <si>
+    <t>Severidad</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>TC-029</t>
+  </si>
+  <si>
+    <t>Límite de intentos de edición del Nombre de perfil (1 vez cada 7 días)</t>
   </si>
   <si>
     <r>
@@ -109,32 +114,32 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: Br-06^</t>
+      <t>Contraseña: tiktok123//; Nombre: Br-06^</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción para editar perfil (símbolo lápiz); 4- Completar el campo “Nombre de perfil”; 5- Seleccionar “Guardar”; 6- Seleccionar “Continuar”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El sistema acepta el formato ingresado y bloquea el campo Nombre durante 7 días</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pasadas las 24hs de establecido el Nombre de Perfil, el sistema volvió a habilitar la edición del mismo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEDIUM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUG: esto se observó manteniendo la app funcionando en segundo plano en el dispositivo movil (Samsung A56), sin apagar ni reiniciar el equipo. Pasadas las 24hs, cuando se volvió a ingresar a la app desde la vista previa de aplicaciones ejecutadas en segundo plano, la pantalla mostró nuevamente el campo Nombre de Perfil con el nombre prestablecido al crear la cuenta nueva.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validar el rechazo de Nombre de usuario con  formato incorrecto: 1 carácter; mayúscula</t>
+    <t>1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción para editar perfil (símbolo lápiz); 4- Completar el campo “Nombre de perfil”; 5- Seleccionar “Guardar”; 6- Seleccionar “Continuar”</t>
+  </si>
+  <si>
+    <t>El sistema acepta el formato ingresado y bloquea el campo Nombre durante 7 días</t>
+  </si>
+  <si>
+    <t>Pasadas las 24hs de establecido el Nombre de Perfil, el sistema volvió a habilitar la edición del mismo</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>BUG: esto se observó manteniendo la app funcionando en segundo plano en el dispositivo movil (Samsung A56), sin apagar ni reiniciar el equipo. Pasadas las 24hs, cuando se volvió a ingresar a la app desde la vista previa de aplicaciones ejecutadas en segundo plano, la pantalla mostró nuevamente el campo Nombre de Perfil con el nombre prestablecido al crear la cuenta nueva.</t>
+  </si>
+  <si>
+    <t>TC-030</t>
+  </si>
+  <si>
+    <t>Validar el rechazo de Nombre de usuario con  formato incorrecto: 1 carácter; mayúscula</t>
   </si>
   <si>
     <r>
@@ -154,47 +159,47 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: B</t>
+      <t>Contraseña: tiktok123//; Nombre: B</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción para editar perfil (símbolo lápiz); 4- Completar el campo “Nombre de perfil”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El sistema rechaza los datos ingresados por incumplimiento de requisitos y debe mostrar claramente las reglas de validación: al menos dos caracteres, sin mayúsculas, sólo puntos y guiones bajos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El sistema rechaza el input pero el mensaje sólo indica  que el nombre no puede tener 1 carácter y no hace mención al resto de las restricciones. El botón “Guardar” queda bloqueado y en color gris.  Las opciones del usuario son: probar nuevamente u omitir la edición</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LOW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUG: el rechazo es validado únicamente por ser &lt;2 caracteres, sin especificar que el uso de mayúscula es inválido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-036</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validar la reanudación de la app al volver desde segundo plano</t>
+    <t>1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción para editar perfil (símbolo lápiz); 4- Completar el campo “Nombre de perfil”</t>
+  </si>
+  <si>
+    <t>El sistema rechaza los datos ingresados por incumplimiento de requisitos y debe mostrar claramente las reglas de validación: al menos dos caracteres, sin mayúsculas, sólo puntos y guiones bajos</t>
+  </si>
+  <si>
+    <t>El sistema rechaza el input pero el mensaje sólo indica  que el nombre no puede tener 1 carácter y no hace mención al resto de las restricciones. El botón “Guardar” queda bloqueado y en color gris.  Las opciones del usuario son: probar nuevamente u omitir la edición</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>BUG: el rechazo es validado únicamente por ser &lt;2 caracteres, sin especificar que el uso de mayúscula es inválido</t>
+  </si>
+  <si>
+    <t>TC-036</t>
+  </si>
+  <si>
+    <t>Validar la reanudación de la app al volver desde segundo plano</t>
   </si>
   <si>
     <t xml:space="preserve"> -</t>
   </si>
   <si>
-    <t xml:space="preserve">1- Ingresar a la app; 2- Navegar el feed; 3- Dejarla ejecutándose en 2do plano; 4- Abrir el menú de aplicaciones recientes en el dispositivo; 5- Volver a la app</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se visualiza la app junto con otras pantallas en 2do plano y al ingresar a la misma debe restaurar la pantalla donde se encontraba el usuario sin perder el estado</t>
+    <t>1- Ingresar a la app; 2- Navegar el feed; 3- Dejarla ejecutándose en 2do plano; 4- Abrir el menú de aplicaciones recientes en el dispositivo; 5- Volver a la app</t>
+  </si>
+  <si>
+    <t>Se visualiza la app junto con otras pantallas en 2do plano y al ingresar a la misma debe restaurar la pantalla donde se encontraba el usuario sin perder el estado</t>
   </si>
   <si>
     <t xml:space="preserve">La vista previa de la app en 2do plano desaparece y la app se comporta como si se hubiese cerrado. </t>
   </si>
   <si>
-    <t xml:space="preserve">HIGH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRITICAL</t>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>CRITICAL</t>
   </si>
   <si>
     <r>
@@ -214,60 +219,42 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Se requirió abrir la app nuevamente, ya sea desde el menú de aplicaciones instaladas en el dispositivo o desde el acceso directo a las últimas aplicaciones utilizadas.</t>
+      <t>Se requirió abrir la app nuevamente, ya sea desde el menú de aplicaciones instaladas en el dispositivo o desde el acceso directo a las últimas aplicaciones utilizadas.</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">TC-037</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validar la visualización de pantalla en “modo oscuro”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1- Ingresar a la app; 2- Ingresar a Configuración; 3- Ingresar a la opción “Pantalla y Accesibilidad”; 4- Seleccionar “modo oscuro”</t>
+    <t>TC-037</t>
+  </si>
+  <si>
+    <t>Validar la visualización de pantalla en “modo oscuro”</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>1- Ingresar a la app; 2- Ingresar a Configuración; 3- Ingresar a la opción “Pantalla y Accesibilidad”; 4- Seleccionar “modo oscuro”</t>
   </si>
   <si>
     <t xml:space="preserve">La pantalla cambia de color, el fondo blanco pasa a negro y esta configuración se mantiene hasta que el usuario decida modificarla </t>
   </si>
   <si>
-    <t xml:space="preserve">El color de fondo aparece en blanco mientras que la configuración de pantalla se encuentra en “modo oscuro”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUG: Durante la ejecución de pruebas, el fondo de la app cambió de color, pasando del modo oscuro al modo claro a pesar de su configuración. El comportamiento no pudo ser reproducido nuevamente para su registro, ya que al ingresar a la configuración de pantalla y visualizar el bug, la app corrigió el mismo automáticamente. Por lo tanto sólo se registra como una observación.</t>
+    <t>El color de fondo aparece en blanco mientras que la configuración de pantalla se encuentra en “modo oscuro”</t>
+  </si>
+  <si>
+    <t>BUG: Durante la ejecución de pruebas, el fondo de la app cambió de color, pasando del modo oscuro al modo claro a pesar de su configuración. El comportamiento no pudo ser reproducido nuevamente para su registro, ya que al ingresar a la configuración de pantalla y visualizar el bug, la app corrigió el mismo automáticamente. Por lo tanto sólo se registra como una observación.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
       <sz val="11"/>
@@ -302,76 +289,52 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -430,60 +393,76 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -515,7 +494,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -539,7 +518,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -599,33 +578,32 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J38"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="29.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="44.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="39.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="50.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="85.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="5" max="5" width="39.21875" customWidth="1"/>
+    <col min="6" max="6" width="50.5546875" customWidth="1"/>
+    <col min="7" max="9" width="11.5546875" customWidth="1"/>
+    <col min="10" max="10" width="85.5546875" customWidth="1"/>
+    <col min="16384" max="16384" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -657,7 +635,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:10" ht="119.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -689,7 +667,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="73.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:10" ht="73.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
@@ -721,7 +699,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="72.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:10" ht="127.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>27</v>
       </c>
@@ -753,7 +731,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="62.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:10" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>36</v>
       </c>
@@ -785,24 +763,19 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="135.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="80.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="103.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="97.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="158.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="156.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="33" ht="135.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="34" ht="80.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="35" ht="103.65" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="36" ht="97.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="37" ht="158.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="38" ht="156.6" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId2" display="breru.qatest@gmail.com"/>
-    <hyperlink ref="C3" r:id="rId3" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="C2" r:id="rId1" display="breru.qatest@gmail.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="C3" r:id="rId2" display="breru.qatest@gmail.com" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <legacyDrawing r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>